<commit_message>
Add Jupyter Notebook for WSDP operations with error handling and WS-Security
- Created a new Jupyter Notebook for interacting with the WSDP (Web Services for the Cadastre) API.
- Implemented installation of the required `zeep` library.
- Added code to list available operations and their parameters.
- Included error handling for SOAP faults during API calls.
- Integrated WS-Security for authentication using UsernameToken.
- Provided hard-coded test values for querying property information.
</commit_message>
<xml_diff>
--- a/PYTHON/DATA_ANALYSIS/VALUO/data_strukturovana/___ALL/1/cadastre_report_6_2024 (3).xlsx
+++ b/PYTHON/DATA_ANALYSIS/VALUO/data_strukturovana/___ALL/1/cadastre_report_6_2024 (3).xlsx
@@ -1,21 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28827"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3ad31658eb0d26ad/Dokumenty/PROG/PYTHON/DATA_ANALYSIS/VALUO/data_strukturovana/___ALL/1/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="13" documentId="11_85AD53BF65A3DE744003782BDAAEDC2DABF39583" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D6D75CE2-9EB2-40B8-B7E1-94533115C155}"/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="61656" windowHeight="25416" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Worksheet" sheetId="1" r:id="rId4"/>
+    <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1" forceFullCalc="1"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Worksheet!$A$1:$P$282</definedName>
+  </definedNames>
+  <calcPr calcId="191029" forceFullCalc="1"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1056">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3384" uniqueCount="1056">
   <si>
     <t>Číslo vkladu</t>
   </si>
@@ -3188,16 +3209,12 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00_-"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -3224,14 +3241,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="0" numFmtId="164" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normální" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -3521,14 +3546,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:P282"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="4" max="4" width="20.77734375" customWidth="1"/>
+    <col min="5" max="5" width="25.5546875" customWidth="1"/>
+    <col min="6" max="6" width="10.33203125" customWidth="1"/>
+    <col min="7" max="7" width="51" customWidth="1"/>
+    <col min="11" max="11" width="38.44140625" customWidth="1"/>
+    <col min="12" max="12" width="178.33203125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:16">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3578,7 +3609,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -3607,7 +3638,7 @@
         <v>23</v>
       </c>
       <c r="J2" s="1">
-        <v>74.0</v>
+        <v>74</v>
       </c>
       <c r="K2" t="s">
         <v>24</v>
@@ -3628,7 +3659,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:16">
+    <row r="3" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>28</v>
       </c>
@@ -3678,7 +3709,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:16">
+    <row r="4" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -3707,7 +3738,7 @@
         <v>23</v>
       </c>
       <c r="J4" s="1">
-        <v>108.0</v>
+        <v>108</v>
       </c>
       <c r="K4" t="s">
         <v>41</v>
@@ -3728,7 +3759,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:16">
+    <row r="5" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>35</v>
       </c>
@@ -3757,7 +3788,7 @@
         <v>23</v>
       </c>
       <c r="J5" s="1">
-        <v>83.0</v>
+        <v>83</v>
       </c>
       <c r="K5" t="s">
         <v>41</v>
@@ -3778,7 +3809,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:16">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>47</v>
       </c>
@@ -3828,7 +3859,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:16">
+    <row r="7" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>47</v>
       </c>
@@ -3878,7 +3909,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:16">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>54</v>
       </c>
@@ -3928,7 +3959,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:16">
+    <row r="9" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>54</v>
       </c>
@@ -3957,7 +3988,7 @@
         <v>23</v>
       </c>
       <c r="J9" s="1">
-        <v>265.0</v>
+        <v>265</v>
       </c>
       <c r="K9" t="s">
         <v>41</v>
@@ -3978,7 +4009,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:16">
+    <row r="10" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>54</v>
       </c>
@@ -4007,7 +4038,7 @@
         <v>23</v>
       </c>
       <c r="J10" s="1">
-        <v>154.0</v>
+        <v>154</v>
       </c>
       <c r="K10" t="s">
         <v>41</v>
@@ -4028,7 +4059,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:16">
+    <row r="11" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>54</v>
       </c>
@@ -4057,7 +4088,7 @@
         <v>23</v>
       </c>
       <c r="J11" s="1">
-        <v>265.0</v>
+        <v>265</v>
       </c>
       <c r="K11" t="s">
         <v>41</v>
@@ -4078,7 +4109,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:16">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>67</v>
       </c>
@@ -4128,7 +4159,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:16">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>72</v>
       </c>
@@ -4178,7 +4209,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:16">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>77</v>
       </c>
@@ -4228,7 +4259,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="1:16">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>81</v>
       </c>
@@ -4278,7 +4309,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:16">
+    <row r="16" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>81</v>
       </c>
@@ -4328,7 +4359,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:16">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>86</v>
       </c>
@@ -4357,7 +4388,7 @@
         <v>23</v>
       </c>
       <c r="J17" s="1">
-        <v>464.0</v>
+        <v>464</v>
       </c>
       <c r="K17" t="s">
         <v>41</v>
@@ -4378,7 +4409,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:16">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>91</v>
       </c>
@@ -4428,7 +4459,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="19" spans="1:16">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>95</v>
       </c>
@@ -4478,7 +4509,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="20" spans="1:16">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>99</v>
       </c>
@@ -4528,7 +4559,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="21" spans="1:16">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>104</v>
       </c>
@@ -4578,7 +4609,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="22" spans="1:16">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>109</v>
       </c>
@@ -4628,7 +4659,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:16">
+    <row r="23" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>113</v>
       </c>
@@ -4657,7 +4688,7 @@
         <v>23</v>
       </c>
       <c r="J23" s="1">
-        <v>9.0</v>
+        <v>9</v>
       </c>
       <c r="K23" t="s">
         <v>41</v>
@@ -4678,7 +4709,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="24" spans="1:16">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>118</v>
       </c>
@@ -4728,7 +4759,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:16">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>123</v>
       </c>
@@ -4778,7 +4809,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="26" spans="1:16">
+    <row r="26" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>128</v>
       </c>
@@ -4807,7 +4838,7 @@
         <v>23</v>
       </c>
       <c r="J26" s="1">
-        <v>387.0</v>
+        <v>387</v>
       </c>
       <c r="K26" t="s">
         <v>41</v>
@@ -4828,7 +4859,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="27" spans="1:16">
+    <row r="27" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>128</v>
       </c>
@@ -4857,7 +4888,7 @@
         <v>23</v>
       </c>
       <c r="J27" s="1">
-        <v>65.0</v>
+        <v>65</v>
       </c>
       <c r="K27" t="s">
         <v>41</v>
@@ -4878,7 +4909,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="28" spans="1:16">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>135</v>
       </c>
@@ -4907,7 +4938,7 @@
         <v>23</v>
       </c>
       <c r="J28" s="1">
-        <v>73.0</v>
+        <v>73</v>
       </c>
       <c r="K28" t="s">
         <v>24</v>
@@ -4928,7 +4959,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="29" spans="1:16">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>140</v>
       </c>
@@ -4978,7 +5009,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="30" spans="1:16">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>144</v>
       </c>
@@ -5028,7 +5059,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="31" spans="1:16">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>148</v>
       </c>
@@ -5057,7 +5088,7 @@
         <v>23</v>
       </c>
       <c r="J31" s="1">
-        <v>30.0</v>
+        <v>30</v>
       </c>
       <c r="K31" t="s">
         <v>24</v>
@@ -5078,7 +5109,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="32" spans="1:16">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>153</v>
       </c>
@@ -5107,7 +5138,7 @@
         <v>23</v>
       </c>
       <c r="J32" s="1">
-        <v>35.62</v>
+        <v>35.619999999999997</v>
       </c>
       <c r="K32" t="s">
         <v>24</v>
@@ -5128,7 +5159,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="33" spans="1:16">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>158</v>
       </c>
@@ -5178,7 +5209,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="34" spans="1:16">
+    <row r="34" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>158</v>
       </c>
@@ -5207,7 +5238,7 @@
         <v>23</v>
       </c>
       <c r="J34" s="1">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="K34" t="s">
         <v>41</v>
@@ -5228,7 +5259,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="35" spans="1:16">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>165</v>
       </c>
@@ -5278,7 +5309,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="36" spans="1:16">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>169</v>
       </c>
@@ -5328,7 +5359,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="37" spans="1:16">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>173</v>
       </c>
@@ -5357,7 +5388,7 @@
         <v>23</v>
       </c>
       <c r="J37" s="1">
-        <v>225.0</v>
+        <v>225</v>
       </c>
       <c r="K37" t="s">
         <v>41</v>
@@ -5378,7 +5409,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="38" spans="1:16">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>178</v>
       </c>
@@ -5407,7 +5438,7 @@
         <v>23</v>
       </c>
       <c r="J38" s="1">
-        <v>74.4</v>
+        <v>74.400000000000006</v>
       </c>
       <c r="K38" t="s">
         <v>24</v>
@@ -5428,7 +5459,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="39" spans="1:16">
+    <row r="39" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>178</v>
       </c>
@@ -5457,7 +5488,7 @@
         <v>23</v>
       </c>
       <c r="J39" s="1">
-        <v>40.37</v>
+        <v>40.369999999999997</v>
       </c>
       <c r="K39" t="s">
         <v>24</v>
@@ -5478,7 +5509,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="40" spans="1:16">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>184</v>
       </c>
@@ -5528,7 +5559,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="41" spans="1:16">
+    <row r="41" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>184</v>
       </c>
@@ -5557,7 +5588,7 @@
         <v>23</v>
       </c>
       <c r="J41" s="1">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="K41" t="s">
         <v>41</v>
@@ -5578,7 +5609,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="42" spans="1:16">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>190</v>
       </c>
@@ -5628,7 +5659,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="43" spans="1:16">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>194</v>
       </c>
@@ -5657,7 +5688,7 @@
         <v>23</v>
       </c>
       <c r="J43" s="1">
-        <v>62.0</v>
+        <v>62</v>
       </c>
       <c r="K43" t="s">
         <v>24</v>
@@ -5678,7 +5709,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="44" spans="1:16">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>199</v>
       </c>
@@ -5728,7 +5759,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="45" spans="1:16">
+    <row r="45" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>199</v>
       </c>
@@ -5757,7 +5788,7 @@
         <v>23</v>
       </c>
       <c r="J45" s="1">
-        <v>11.0</v>
+        <v>11</v>
       </c>
       <c r="K45" t="s">
         <v>41</v>
@@ -5778,7 +5809,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="46" spans="1:16">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>205</v>
       </c>
@@ -5828,7 +5859,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="47" spans="1:16">
+    <row r="47" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>205</v>
       </c>
@@ -5857,7 +5888,7 @@
         <v>23</v>
       </c>
       <c r="J47" s="1">
-        <v>14.0</v>
+        <v>14</v>
       </c>
       <c r="K47" t="s">
         <v>41</v>
@@ -5878,7 +5909,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="48" spans="1:16">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>211</v>
       </c>
@@ -5928,7 +5959,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="49" spans="1:16">
+    <row r="49" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>215</v>
       </c>
@@ -5957,7 +5988,7 @@
         <v>23</v>
       </c>
       <c r="J49" s="1">
-        <v>7.0</v>
+        <v>7</v>
       </c>
       <c r="K49" t="s">
         <v>41</v>
@@ -5978,7 +6009,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="50" spans="1:16">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>220</v>
       </c>
@@ -6028,7 +6059,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="51" spans="1:16">
+    <row r="51" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>220</v>
       </c>
@@ -6078,7 +6109,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="52" spans="1:16">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>224</v>
       </c>
@@ -6107,7 +6138,7 @@
         <v>23</v>
       </c>
       <c r="J52" s="1">
-        <v>37.0</v>
+        <v>37</v>
       </c>
       <c r="K52" t="s">
         <v>24</v>
@@ -6128,7 +6159,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="53" spans="1:16">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>228</v>
       </c>
@@ -6178,7 +6209,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="54" spans="1:16">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>233</v>
       </c>
@@ -6228,7 +6259,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="55" spans="1:16">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>238</v>
       </c>
@@ -6278,7 +6309,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="56" spans="1:16">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>242</v>
       </c>
@@ -6328,7 +6359,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="57" spans="1:16">
+    <row r="57" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>246</v>
       </c>
@@ -6378,7 +6409,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="58" spans="1:16">
+    <row r="58" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>251</v>
       </c>
@@ -6428,7 +6459,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="59" spans="1:16">
+    <row r="59" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>255</v>
       </c>
@@ -6478,7 +6509,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="60" spans="1:16">
+    <row r="60" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>255</v>
       </c>
@@ -6507,7 +6538,7 @@
         <v>23</v>
       </c>
       <c r="J60" s="1">
-        <v>15704.0</v>
+        <v>15704</v>
       </c>
       <c r="K60" t="s">
         <v>260</v>
@@ -6528,7 +6559,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="61" spans="1:16">
+    <row r="61" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>255</v>
       </c>
@@ -6557,7 +6588,7 @@
         <v>23</v>
       </c>
       <c r="J61" s="1">
-        <v>149.0</v>
+        <v>149</v>
       </c>
       <c r="K61" t="s">
         <v>41</v>
@@ -6578,7 +6609,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="62" spans="1:16">
+    <row r="62" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>255</v>
       </c>
@@ -6607,7 +6638,7 @@
         <v>23</v>
       </c>
       <c r="J62" s="1">
-        <v>82.0</v>
+        <v>82</v>
       </c>
       <c r="K62" t="s">
         <v>41</v>
@@ -6628,7 +6659,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="63" spans="1:16">
+    <row r="63" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>255</v>
       </c>
@@ -6657,7 +6688,7 @@
         <v>23</v>
       </c>
       <c r="J63" s="1">
-        <v>73.0</v>
+        <v>73</v>
       </c>
       <c r="K63" t="s">
         <v>41</v>
@@ -6678,7 +6709,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="64" spans="1:16">
+    <row r="64" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>255</v>
       </c>
@@ -6707,7 +6738,7 @@
         <v>23</v>
       </c>
       <c r="J64" s="1">
-        <v>832.0</v>
+        <v>832</v>
       </c>
       <c r="K64" t="s">
         <v>41</v>
@@ -6728,7 +6759,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="65" spans="1:16">
+    <row r="65" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>255</v>
       </c>
@@ -6757,7 +6788,7 @@
         <v>23</v>
       </c>
       <c r="J65" s="1">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="K65" t="s">
         <v>41</v>
@@ -6778,7 +6809,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="66" spans="1:16">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>273</v>
       </c>
@@ -6828,7 +6859,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="67" spans="1:16">
+    <row r="67" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>277</v>
       </c>
@@ -6857,7 +6888,7 @@
         <v>23</v>
       </c>
       <c r="J67" s="1">
-        <v>263.0</v>
+        <v>263</v>
       </c>
       <c r="K67" t="s">
         <v>41</v>
@@ -6878,7 +6909,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="68" spans="1:16">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>282</v>
       </c>
@@ -6928,7 +6959,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="69" spans="1:16">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>282</v>
       </c>
@@ -6978,7 +7009,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="70" spans="1:16">
+    <row r="70" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>288</v>
       </c>
@@ -7007,7 +7038,7 @@
         <v>23</v>
       </c>
       <c r="J70" s="1">
-        <v>21.0</v>
+        <v>21</v>
       </c>
       <c r="K70" t="s">
         <v>41</v>
@@ -7028,7 +7059,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="71" spans="1:16">
+    <row r="71" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>288</v>
       </c>
@@ -7057,7 +7088,7 @@
         <v>23</v>
       </c>
       <c r="J71" s="1">
-        <v>21.0</v>
+        <v>21</v>
       </c>
       <c r="K71" t="s">
         <v>41</v>
@@ -7078,7 +7109,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="72" spans="1:16">
+    <row r="72" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>295</v>
       </c>
@@ -7120,7 +7151,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="73" spans="1:16">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>299</v>
       </c>
@@ -7170,7 +7201,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="74" spans="1:16">
+    <row r="74" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>303</v>
       </c>
@@ -7220,7 +7251,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="75" spans="1:16">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>308</v>
       </c>
@@ -7270,7 +7301,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="76" spans="1:16">
+    <row r="76" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>308</v>
       </c>
@@ -7320,7 +7351,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="77" spans="1:16">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>312</v>
       </c>
@@ -7349,7 +7380,7 @@
         <v>23</v>
       </c>
       <c r="J77" s="1">
-        <v>64.4</v>
+        <v>64.400000000000006</v>
       </c>
       <c r="K77" t="s">
         <v>24</v>
@@ -7370,7 +7401,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="78" spans="1:16">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>316</v>
       </c>
@@ -7420,7 +7451,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="79" spans="1:16">
+    <row r="79" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>316</v>
       </c>
@@ -7449,7 +7480,7 @@
         <v>23</v>
       </c>
       <c r="J79" s="1">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="K79" t="s">
         <v>41</v>
@@ -7470,7 +7501,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="80" spans="1:16">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>322</v>
       </c>
@@ -7520,7 +7551,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="81" spans="1:16">
+    <row r="81" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>322</v>
       </c>
@@ -7570,7 +7601,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="82" spans="1:16">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>326</v>
       </c>
@@ -7620,7 +7651,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="83" spans="1:16">
+    <row r="83" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>326</v>
       </c>
@@ -7649,7 +7680,7 @@
         <v>23</v>
       </c>
       <c r="J83" s="1">
-        <v>208.0</v>
+        <v>208</v>
       </c>
       <c r="K83" t="s">
         <v>41</v>
@@ -7670,7 +7701,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="84" spans="1:16">
+    <row r="84" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>326</v>
       </c>
@@ -7699,7 +7730,7 @@
         <v>23</v>
       </c>
       <c r="J84" s="1">
-        <v>184.0</v>
+        <v>184</v>
       </c>
       <c r="K84" t="s">
         <v>41</v>
@@ -7720,7 +7751,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="85" spans="1:16">
+    <row r="85" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>335</v>
       </c>
@@ -7749,7 +7780,7 @@
         <v>23</v>
       </c>
       <c r="J85" s="1">
-        <v>157.0</v>
+        <v>157</v>
       </c>
       <c r="K85" t="s">
         <v>41</v>
@@ -7770,7 +7801,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="86" spans="1:16">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>340</v>
       </c>
@@ -7820,7 +7851,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="87" spans="1:16">
+    <row r="87" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>344</v>
       </c>
@@ -7849,7 +7880,7 @@
         <v>23</v>
       </c>
       <c r="J87" s="1">
-        <v>19.0</v>
+        <v>19</v>
       </c>
       <c r="K87" t="s">
         <v>41</v>
@@ -7870,7 +7901,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="88" spans="1:16">
+    <row r="88" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>349</v>
       </c>
@@ -7920,7 +7951,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="89" spans="1:16">
+    <row r="89" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>354</v>
       </c>
@@ -7970,7 +8001,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="90" spans="1:16">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>358</v>
       </c>
@@ -8020,7 +8051,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="91" spans="1:16">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>363</v>
       </c>
@@ -8070,7 +8101,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="92" spans="1:16">
+    <row r="92" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>367</v>
       </c>
@@ -8099,7 +8130,7 @@
         <v>23</v>
       </c>
       <c r="J92" s="1">
-        <v>182.0</v>
+        <v>182</v>
       </c>
       <c r="K92" t="s">
         <v>41</v>
@@ -8120,7 +8151,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="93" spans="1:16">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>372</v>
       </c>
@@ -8170,7 +8201,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="94" spans="1:16">
+    <row r="94" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>376</v>
       </c>
@@ -8199,7 +8230,7 @@
         <v>23</v>
       </c>
       <c r="J94" s="1">
-        <v>2407.0</v>
+        <v>2407</v>
       </c>
       <c r="K94" t="s">
         <v>41</v>
@@ -8220,7 +8251,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="95" spans="1:16">
+    <row r="95" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>376</v>
       </c>
@@ -8249,7 +8280,7 @@
         <v>23</v>
       </c>
       <c r="J95" s="1">
-        <v>18318.0</v>
+        <v>18318</v>
       </c>
       <c r="K95" t="s">
         <v>41</v>
@@ -8270,7 +8301,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="96" spans="1:16">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>384</v>
       </c>
@@ -8299,7 +8330,7 @@
         <v>23</v>
       </c>
       <c r="J96" s="1">
-        <v>276.0</v>
+        <v>276</v>
       </c>
       <c r="K96" t="s">
         <v>41</v>
@@ -8320,7 +8351,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="97" spans="1:16">
+    <row r="97" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>384</v>
       </c>
@@ -8349,7 +8380,7 @@
         <v>23</v>
       </c>
       <c r="J97" s="1">
-        <v>253.0</v>
+        <v>253</v>
       </c>
       <c r="K97" t="s">
         <v>41</v>
@@ -8370,7 +8401,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="98" spans="1:16">
+    <row r="98" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>391</v>
       </c>
@@ -8420,7 +8451,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="99" spans="1:16">
+    <row r="99" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>396</v>
       </c>
@@ -8470,7 +8501,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="100" spans="1:16">
+    <row r="100" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>400</v>
       </c>
@@ -8520,7 +8551,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="101" spans="1:16">
+    <row r="101" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>404</v>
       </c>
@@ -8570,7 +8601,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="102" spans="1:16">
+    <row r="102" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>408</v>
       </c>
@@ -8599,7 +8630,7 @@
         <v>23</v>
       </c>
       <c r="J102" s="1">
-        <v>42.0</v>
+        <v>42</v>
       </c>
       <c r="K102" t="s">
         <v>24</v>
@@ -8620,7 +8651,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="103" spans="1:16">
+    <row r="103" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>413</v>
       </c>
@@ -8649,7 +8680,7 @@
         <v>23</v>
       </c>
       <c r="J103" s="1">
-        <v>256.0</v>
+        <v>256</v>
       </c>
       <c r="K103" t="s">
         <v>41</v>
@@ -8670,7 +8701,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="104" spans="1:16">
+    <row r="104" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>419</v>
       </c>
@@ -8720,7 +8751,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="105" spans="1:16">
+    <row r="105" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>419</v>
       </c>
@@ -8749,7 +8780,7 @@
         <v>23</v>
       </c>
       <c r="J105" s="1">
-        <v>88.0</v>
+        <v>88</v>
       </c>
       <c r="K105" t="s">
         <v>41</v>
@@ -8770,7 +8801,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="106" spans="1:16">
+    <row r="106" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>427</v>
       </c>
@@ -8820,7 +8851,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="107" spans="1:16">
+    <row r="107" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>432</v>
       </c>
@@ -8870,7 +8901,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="108" spans="1:16">
+    <row r="108" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>436</v>
       </c>
@@ -8899,7 +8930,7 @@
         <v>23</v>
       </c>
       <c r="J108" s="1">
-        <v>37.0</v>
+        <v>37</v>
       </c>
       <c r="K108" t="s">
         <v>24</v>
@@ -8920,7 +8951,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="109" spans="1:16">
+    <row r="109" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>440</v>
       </c>
@@ -8970,7 +9001,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="110" spans="1:16">
+    <row r="110" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>444</v>
       </c>
@@ -8999,7 +9030,7 @@
         <v>23</v>
       </c>
       <c r="J110" s="1">
-        <v>24.0</v>
+        <v>24</v>
       </c>
       <c r="K110" t="s">
         <v>41</v>
@@ -9020,7 +9051,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="111" spans="1:16">
+    <row r="111" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>449</v>
       </c>
@@ -9070,7 +9101,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="112" spans="1:16">
+    <row r="112" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>454</v>
       </c>
@@ -9099,7 +9130,7 @@
         <v>23</v>
       </c>
       <c r="J112" s="1">
-        <v>80.1</v>
+        <v>80.099999999999994</v>
       </c>
       <c r="K112" t="s">
         <v>24</v>
@@ -9120,7 +9151,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="113" spans="1:16">
+    <row r="113" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>454</v>
       </c>
@@ -9149,7 +9180,7 @@
         <v>23</v>
       </c>
       <c r="J113" s="1">
-        <v>375.0</v>
+        <v>375</v>
       </c>
       <c r="K113" t="s">
         <v>41</v>
@@ -9170,7 +9201,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="114" spans="1:16">
+    <row r="114" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>460</v>
       </c>
@@ -9212,7 +9243,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="115" spans="1:16">
+    <row r="115" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>464</v>
       </c>
@@ -9241,7 +9272,7 @@
         <v>23</v>
       </c>
       <c r="J115" s="1">
-        <v>37.0</v>
+        <v>37</v>
       </c>
       <c r="K115" t="s">
         <v>24</v>
@@ -9262,7 +9293,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="116" spans="1:16">
+    <row r="116" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>464</v>
       </c>
@@ -9291,7 +9322,7 @@
         <v>23</v>
       </c>
       <c r="J116" s="1">
-        <v>11.0</v>
+        <v>11</v>
       </c>
       <c r="K116" t="s">
         <v>41</v>
@@ -9312,7 +9343,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="117" spans="1:16">
+    <row r="117" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>470</v>
       </c>
@@ -9362,7 +9393,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="118" spans="1:16">
+    <row r="118" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>474</v>
       </c>
@@ -9412,7 +9443,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="119" spans="1:16">
+    <row r="119" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>479</v>
       </c>
@@ -9441,7 +9472,7 @@
         <v>23</v>
       </c>
       <c r="J119" s="1">
-        <v>254.0</v>
+        <v>254</v>
       </c>
       <c r="K119" t="s">
         <v>41</v>
@@ -9462,7 +9493,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="120" spans="1:16">
+    <row r="120" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>479</v>
       </c>
@@ -9491,7 +9522,7 @@
         <v>23</v>
       </c>
       <c r="J120" s="1">
-        <v>329.0</v>
+        <v>329</v>
       </c>
       <c r="K120" t="s">
         <v>41</v>
@@ -9512,7 +9543,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="121" spans="1:16">
+    <row r="121" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>486</v>
       </c>
@@ -9562,7 +9593,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="122" spans="1:16">
+    <row r="122" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>490</v>
       </c>
@@ -9612,7 +9643,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="123" spans="1:16">
+    <row r="123" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>493</v>
       </c>
@@ -9641,7 +9672,7 @@
         <v>23</v>
       </c>
       <c r="J123" s="1">
-        <v>98.0</v>
+        <v>98</v>
       </c>
       <c r="K123" t="s">
         <v>41</v>
@@ -9662,7 +9693,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="124" spans="1:16">
+    <row r="124" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>499</v>
       </c>
@@ -9712,7 +9743,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="125" spans="1:16">
+    <row r="125" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>504</v>
       </c>
@@ -9741,7 +9772,7 @@
         <v>23</v>
       </c>
       <c r="J125" s="1">
-        <v>72.0</v>
+        <v>72</v>
       </c>
       <c r="K125" t="s">
         <v>24</v>
@@ -9762,7 +9793,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="126" spans="1:16">
+    <row r="126" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>509</v>
       </c>
@@ -9812,7 +9843,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="127" spans="1:16">
+    <row r="127" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>513</v>
       </c>
@@ -9862,7 +9893,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="128" spans="1:16">
+    <row r="128" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>517</v>
       </c>
@@ -9912,7 +9943,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="129" spans="1:16">
+    <row r="129" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>517</v>
       </c>
@@ -9962,7 +9993,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="130" spans="1:16">
+    <row r="130" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>517</v>
       </c>
@@ -10012,7 +10043,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="131" spans="1:16">
+    <row r="131" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>522</v>
       </c>
@@ -10062,7 +10093,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="132" spans="1:16">
+    <row r="132" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>526</v>
       </c>
@@ -10112,7 +10143,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="133" spans="1:16">
+    <row r="133" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>526</v>
       </c>
@@ -10141,7 +10172,7 @@
         <v>23</v>
       </c>
       <c r="J133" s="1">
-        <v>132.0</v>
+        <v>132</v>
       </c>
       <c r="K133" t="s">
         <v>41</v>
@@ -10162,7 +10193,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="134" spans="1:16">
+    <row r="134" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>526</v>
       </c>
@@ -10191,7 +10222,7 @@
         <v>23</v>
       </c>
       <c r="J134" s="1">
-        <v>7.0</v>
+        <v>7</v>
       </c>
       <c r="K134" t="s">
         <v>41</v>
@@ -10212,7 +10243,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="135" spans="1:16">
+    <row r="135" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>526</v>
       </c>
@@ -10241,7 +10272,7 @@
         <v>23</v>
       </c>
       <c r="J135" s="1">
-        <v>229.0</v>
+        <v>229</v>
       </c>
       <c r="K135" t="s">
         <v>41</v>
@@ -10262,7 +10293,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="136" spans="1:16">
+    <row r="136" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>526</v>
       </c>
@@ -10291,7 +10322,7 @@
         <v>23</v>
       </c>
       <c r="J136" s="1">
-        <v>96.0</v>
+        <v>96</v>
       </c>
       <c r="K136" t="s">
         <v>41</v>
@@ -10312,7 +10343,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="137" spans="1:16">
+    <row r="137" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>526</v>
       </c>
@@ -10341,7 +10372,7 @@
         <v>23</v>
       </c>
       <c r="J137" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="K137" t="s">
         <v>41</v>
@@ -10362,7 +10393,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="138" spans="1:16">
+    <row r="138" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>526</v>
       </c>
@@ -10391,7 +10422,7 @@
         <v>23</v>
       </c>
       <c r="J138" s="1">
-        <v>91.0</v>
+        <v>91</v>
       </c>
       <c r="K138" t="s">
         <v>41</v>
@@ -10412,7 +10443,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="139" spans="1:16">
+    <row r="139" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>526</v>
       </c>
@@ -10441,7 +10472,7 @@
         <v>23</v>
       </c>
       <c r="J139" s="1">
-        <v>47.0</v>
+        <v>47</v>
       </c>
       <c r="K139" t="s">
         <v>41</v>
@@ -10462,7 +10493,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="140" spans="1:16">
+    <row r="140" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>526</v>
       </c>
@@ -10491,7 +10522,7 @@
         <v>23</v>
       </c>
       <c r="J140" s="1">
-        <v>308.0</v>
+        <v>308</v>
       </c>
       <c r="K140" t="s">
         <v>41</v>
@@ -10512,7 +10543,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="141" spans="1:16">
+    <row r="141" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>548</v>
       </c>
@@ -10562,7 +10593,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="142" spans="1:16">
+    <row r="142" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>552</v>
       </c>
@@ -10591,7 +10622,7 @@
         <v>23</v>
       </c>
       <c r="J142" s="1">
-        <v>211.0</v>
+        <v>211</v>
       </c>
       <c r="K142" t="s">
         <v>41</v>
@@ -10612,7 +10643,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="143" spans="1:16">
+    <row r="143" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>558</v>
       </c>
@@ -10662,7 +10693,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="144" spans="1:16">
+    <row r="144" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>562</v>
       </c>
@@ -10712,7 +10743,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="145" spans="1:16">
+    <row r="145" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>566</v>
       </c>
@@ -10762,7 +10793,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="146" spans="1:16">
+    <row r="146" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>570</v>
       </c>
@@ -10791,7 +10822,7 @@
         <v>23</v>
       </c>
       <c r="J146" s="1">
-        <v>13.0</v>
+        <v>13</v>
       </c>
       <c r="K146" t="s">
         <v>41</v>
@@ -10812,7 +10843,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="147" spans="1:16">
+    <row r="147" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>575</v>
       </c>
@@ -10862,7 +10893,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="148" spans="1:16">
+    <row r="148" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>579</v>
       </c>
@@ -10912,7 +10943,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="149" spans="1:16">
+    <row r="149" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>583</v>
       </c>
@@ -10962,7 +10993,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="150" spans="1:16">
+    <row r="150" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>587</v>
       </c>
@@ -10991,7 +11022,7 @@
         <v>23</v>
       </c>
       <c r="J150" s="1">
-        <v>75.4</v>
+        <v>75.400000000000006</v>
       </c>
       <c r="K150" t="s">
         <v>24</v>
@@ -11012,7 +11043,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="151" spans="1:16">
+    <row r="151" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>591</v>
       </c>
@@ -11062,7 +11093,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="152" spans="1:16">
+    <row r="152" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>595</v>
       </c>
@@ -11091,7 +11122,7 @@
         <v>23</v>
       </c>
       <c r="J152" s="1">
-        <v>19.0</v>
+        <v>19</v>
       </c>
       <c r="K152" t="s">
         <v>41</v>
@@ -11112,7 +11143,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="153" spans="1:16">
+    <row r="153" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>595</v>
       </c>
@@ -11141,7 +11172,7 @@
         <v>23</v>
       </c>
       <c r="J153" s="1">
-        <v>77.0</v>
+        <v>77</v>
       </c>
       <c r="K153" t="s">
         <v>41</v>
@@ -11162,7 +11193,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="154" spans="1:16">
+    <row r="154" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>595</v>
       </c>
@@ -11191,7 +11222,7 @@
         <v>23</v>
       </c>
       <c r="J154" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="K154" t="s">
         <v>41</v>
@@ -11212,7 +11243,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="155" spans="1:16">
+    <row r="155" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>604</v>
       </c>
@@ -11241,7 +11272,7 @@
         <v>23</v>
       </c>
       <c r="J155" s="1">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="K155" t="s">
         <v>41</v>
@@ -11262,7 +11293,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="156" spans="1:16">
+    <row r="156" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>609</v>
       </c>
@@ -11291,7 +11322,7 @@
         <v>23</v>
       </c>
       <c r="J156" s="1">
-        <v>29.0</v>
+        <v>29</v>
       </c>
       <c r="K156" t="s">
         <v>24</v>
@@ -11312,7 +11343,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="157" spans="1:16">
+    <row r="157" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>614</v>
       </c>
@@ -11362,7 +11393,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="158" spans="1:16">
+    <row r="158" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>618</v>
       </c>
@@ -11412,7 +11443,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="159" spans="1:16">
+    <row r="159" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>622</v>
       </c>
@@ -11462,7 +11493,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="160" spans="1:16">
+    <row r="160" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>626</v>
       </c>
@@ -11512,7 +11543,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="161" spans="1:16">
+    <row r="161" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>630</v>
       </c>
@@ -11562,7 +11593,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="162" spans="1:16">
+    <row r="162" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>630</v>
       </c>
@@ -11591,7 +11622,7 @@
         <v>23</v>
       </c>
       <c r="J162" s="1">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="K162" t="s">
         <v>41</v>
@@ -11612,7 +11643,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="163" spans="1:16">
+    <row r="163" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>630</v>
       </c>
@@ -11641,7 +11672,7 @@
         <v>23</v>
       </c>
       <c r="J163" s="1">
-        <v>1181.0</v>
+        <v>1181</v>
       </c>
       <c r="K163" t="s">
         <v>41</v>
@@ -11662,7 +11693,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="164" spans="1:16">
+    <row r="164" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>630</v>
       </c>
@@ -11691,7 +11722,7 @@
         <v>23</v>
       </c>
       <c r="J164" s="1">
-        <v>525.0</v>
+        <v>525</v>
       </c>
       <c r="K164" t="s">
         <v>41</v>
@@ -11712,7 +11743,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="165" spans="1:16">
+    <row r="165" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>630</v>
       </c>
@@ -11741,7 +11772,7 @@
         <v>23</v>
       </c>
       <c r="J165" s="1">
-        <v>17.0</v>
+        <v>17</v>
       </c>
       <c r="K165" t="s">
         <v>41</v>
@@ -11762,7 +11793,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="166" spans="1:16">
+    <row r="166" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>643</v>
       </c>
@@ -11791,7 +11822,7 @@
         <v>23</v>
       </c>
       <c r="J166" s="1">
-        <v>12914.0</v>
+        <v>12914</v>
       </c>
       <c r="K166" t="s">
         <v>41</v>
@@ -11812,7 +11843,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="167" spans="1:16">
+    <row r="167" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>643</v>
       </c>
@@ -11841,7 +11872,7 @@
         <v>23</v>
       </c>
       <c r="J167" s="1">
-        <v>2758.0</v>
+        <v>2758</v>
       </c>
       <c r="K167" t="s">
         <v>41</v>
@@ -11862,7 +11893,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="168" spans="1:16">
+    <row r="168" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>643</v>
       </c>
@@ -11891,7 +11922,7 @@
         <v>23</v>
       </c>
       <c r="J168" s="1">
-        <v>12366.0</v>
+        <v>12366</v>
       </c>
       <c r="K168" t="s">
         <v>41</v>
@@ -11912,7 +11943,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="169" spans="1:16">
+    <row r="169" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>643</v>
       </c>
@@ -11941,7 +11972,7 @@
         <v>23</v>
       </c>
       <c r="J169" s="1">
-        <v>192.0</v>
+        <v>192</v>
       </c>
       <c r="K169" t="s">
         <v>41</v>
@@ -11962,7 +11993,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="170" spans="1:16">
+    <row r="170" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>643</v>
       </c>
@@ -11991,7 +12022,7 @@
         <v>23</v>
       </c>
       <c r="J170" s="1">
-        <v>7166.0</v>
+        <v>7166</v>
       </c>
       <c r="K170" t="s">
         <v>41</v>
@@ -12012,7 +12043,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="171" spans="1:16">
+    <row r="171" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>643</v>
       </c>
@@ -12041,7 +12072,7 @@
         <v>23</v>
       </c>
       <c r="J171" s="1">
-        <v>10238.0</v>
+        <v>10238</v>
       </c>
       <c r="K171" t="s">
         <v>41</v>
@@ -12062,7 +12093,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="172" spans="1:16">
+    <row r="172" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>643</v>
       </c>
@@ -12091,7 +12122,7 @@
         <v>23</v>
       </c>
       <c r="J172" s="1">
-        <v>9.0</v>
+        <v>9</v>
       </c>
       <c r="K172" t="s">
         <v>41</v>
@@ -12112,7 +12143,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="173" spans="1:16">
+    <row r="173" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>643</v>
       </c>
@@ -12141,7 +12172,7 @@
         <v>23</v>
       </c>
       <c r="J173" s="1">
-        <v>429.0</v>
+        <v>429</v>
       </c>
       <c r="K173" t="s">
         <v>41</v>
@@ -12162,7 +12193,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="174" spans="1:16">
+    <row r="174" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>643</v>
       </c>
@@ -12191,7 +12222,7 @@
         <v>23</v>
       </c>
       <c r="J174" s="1">
-        <v>54.0</v>
+        <v>54</v>
       </c>
       <c r="K174" t="s">
         <v>41</v>
@@ -12212,7 +12243,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="175" spans="1:16">
+    <row r="175" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>643</v>
       </c>
@@ -12241,7 +12272,7 @@
         <v>23</v>
       </c>
       <c r="J175" s="1">
-        <v>17.0</v>
+        <v>17</v>
       </c>
       <c r="K175" t="s">
         <v>41</v>
@@ -12262,7 +12293,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="176" spans="1:16">
+    <row r="176" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>643</v>
       </c>
@@ -12291,7 +12322,7 @@
         <v>23</v>
       </c>
       <c r="J176" s="1">
-        <v>71.0</v>
+        <v>71</v>
       </c>
       <c r="K176" t="s">
         <v>41</v>
@@ -12312,7 +12343,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="177" spans="1:16">
+    <row r="177" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>669</v>
       </c>
@@ -12341,7 +12372,7 @@
         <v>23</v>
       </c>
       <c r="J177" s="1">
-        <v>430.0</v>
+        <v>430</v>
       </c>
       <c r="K177" t="s">
         <v>41</v>
@@ -12362,7 +12393,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="178" spans="1:16">
+    <row r="178" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>674</v>
       </c>
@@ -12412,7 +12443,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="179" spans="1:16">
+    <row r="179" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>679</v>
       </c>
@@ -12441,7 +12472,7 @@
         <v>23</v>
       </c>
       <c r="J179" s="1">
-        <v>118.0</v>
+        <v>118</v>
       </c>
       <c r="K179" t="s">
         <v>41</v>
@@ -12462,7 +12493,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="180" spans="1:16">
+    <row r="180" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>684</v>
       </c>
@@ -12491,7 +12522,7 @@
         <v>23</v>
       </c>
       <c r="J180" s="1">
-        <v>518.0</v>
+        <v>518</v>
       </c>
       <c r="K180" t="s">
         <v>41</v>
@@ -12512,7 +12543,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="181" spans="1:16">
+    <row r="181" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>684</v>
       </c>
@@ -12541,7 +12572,7 @@
         <v>23</v>
       </c>
       <c r="J181" s="1">
-        <v>305.0</v>
+        <v>305</v>
       </c>
       <c r="K181" t="s">
         <v>41</v>
@@ -12562,7 +12593,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="182" spans="1:16">
+    <row r="182" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>684</v>
       </c>
@@ -12591,7 +12622,7 @@
         <v>23</v>
       </c>
       <c r="J182" s="1">
-        <v>1289.0</v>
+        <v>1289</v>
       </c>
       <c r="K182" t="s">
         <v>41</v>
@@ -12612,7 +12643,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="183" spans="1:16">
+    <row r="183" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>694</v>
       </c>
@@ -12662,7 +12693,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="184" spans="1:16">
+    <row r="184" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>694</v>
       </c>
@@ -12691,7 +12722,7 @@
         <v>23</v>
       </c>
       <c r="J184" s="1">
-        <v>125.0</v>
+        <v>125</v>
       </c>
       <c r="K184" t="s">
         <v>41</v>
@@ -12712,7 +12743,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="185" spans="1:16">
+    <row r="185" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>701</v>
       </c>
@@ -12762,7 +12793,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="186" spans="1:16">
+    <row r="186" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>705</v>
       </c>
@@ -12812,7 +12843,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="187" spans="1:16">
+    <row r="187" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>710</v>
       </c>
@@ -12841,7 +12872,7 @@
         <v>23</v>
       </c>
       <c r="J187" s="1">
-        <v>50.0</v>
+        <v>50</v>
       </c>
       <c r="K187" t="s">
         <v>24</v>
@@ -12862,7 +12893,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="188" spans="1:16">
+    <row r="188" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>710</v>
       </c>
@@ -12891,7 +12922,7 @@
         <v>23</v>
       </c>
       <c r="J188" s="1">
-        <v>213.0</v>
+        <v>213</v>
       </c>
       <c r="K188" t="s">
         <v>41</v>
@@ -12912,7 +12943,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="189" spans="1:16">
+    <row r="189" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>710</v>
       </c>
@@ -12941,7 +12972,7 @@
         <v>23</v>
       </c>
       <c r="J189" s="1">
-        <v>200.0</v>
+        <v>200</v>
       </c>
       <c r="K189" t="s">
         <v>41</v>
@@ -12962,7 +12993,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="190" spans="1:16">
+    <row r="190" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>710</v>
       </c>
@@ -12991,7 +13022,7 @@
         <v>23</v>
       </c>
       <c r="J190" s="1">
-        <v>207.0</v>
+        <v>207</v>
       </c>
       <c r="K190" t="s">
         <v>41</v>
@@ -13012,7 +13043,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="191" spans="1:16">
+    <row r="191" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>720</v>
       </c>
@@ -13041,7 +13072,7 @@
         <v>23</v>
       </c>
       <c r="J191" s="1">
-        <v>78.6</v>
+        <v>78.599999999999994</v>
       </c>
       <c r="K191" t="s">
         <v>24</v>
@@ -13062,7 +13093,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="192" spans="1:16">
+    <row r="192" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>725</v>
       </c>
@@ -13112,7 +13143,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="193" spans="1:16">
+    <row r="193" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>729</v>
       </c>
@@ -13141,7 +13172,7 @@
         <v>23</v>
       </c>
       <c r="J193" s="1">
-        <v>232.0</v>
+        <v>232</v>
       </c>
       <c r="K193" t="s">
         <v>41</v>
@@ -13162,7 +13193,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="194" spans="1:16">
+    <row r="194" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>729</v>
       </c>
@@ -13191,7 +13222,7 @@
         <v>23</v>
       </c>
       <c r="J194" s="1">
-        <v>232.0</v>
+        <v>232</v>
       </c>
       <c r="K194" t="s">
         <v>41</v>
@@ -13212,7 +13243,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="195" spans="1:16">
+    <row r="195" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>729</v>
       </c>
@@ -13241,7 +13272,7 @@
         <v>23</v>
       </c>
       <c r="J195" s="1">
-        <v>223.0</v>
+        <v>223</v>
       </c>
       <c r="K195" t="s">
         <v>41</v>
@@ -13262,7 +13293,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="196" spans="1:16">
+    <row r="196" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>737</v>
       </c>
@@ -13291,7 +13322,7 @@
         <v>23</v>
       </c>
       <c r="J196" s="1">
-        <v>614.0</v>
+        <v>614</v>
       </c>
       <c r="K196" t="s">
         <v>41</v>
@@ -13312,7 +13343,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="197" spans="1:16">
+    <row r="197" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>737</v>
       </c>
@@ -13341,7 +13372,7 @@
         <v>23</v>
       </c>
       <c r="J197" s="1">
-        <v>1988.0</v>
+        <v>1988</v>
       </c>
       <c r="K197" t="s">
         <v>41</v>
@@ -13362,7 +13393,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="198" spans="1:16">
+    <row r="198" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>737</v>
       </c>
@@ -13391,7 +13422,7 @@
         <v>23</v>
       </c>
       <c r="J198" s="1">
-        <v>352.0</v>
+        <v>352</v>
       </c>
       <c r="K198" t="s">
         <v>41</v>
@@ -13412,7 +13443,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="199" spans="1:16">
+    <row r="199" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>737</v>
       </c>
@@ -13441,7 +13472,7 @@
         <v>23</v>
       </c>
       <c r="J199" s="1">
-        <v>207.0</v>
+        <v>207</v>
       </c>
       <c r="K199" t="s">
         <v>41</v>
@@ -13462,7 +13493,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="200" spans="1:16">
+    <row r="200" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>749</v>
       </c>
@@ -13512,7 +13543,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="201" spans="1:16">
+    <row r="201" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>753</v>
       </c>
@@ -13541,7 +13572,7 @@
         <v>23</v>
       </c>
       <c r="J201" s="1">
-        <v>583.0</v>
+        <v>583</v>
       </c>
       <c r="K201" t="s">
         <v>41</v>
@@ -13562,7 +13593,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="202" spans="1:16">
+    <row r="202" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>753</v>
       </c>
@@ -13591,7 +13622,7 @@
         <v>23</v>
       </c>
       <c r="J202" s="1">
-        <v>54.0</v>
+        <v>54</v>
       </c>
       <c r="K202" t="s">
         <v>41</v>
@@ -13612,7 +13643,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="203" spans="1:16">
+    <row r="203" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>753</v>
       </c>
@@ -13641,7 +13672,7 @@
         <v>23</v>
       </c>
       <c r="J203" s="1">
-        <v>105.0</v>
+        <v>105</v>
       </c>
       <c r="K203" t="s">
         <v>41</v>
@@ -13662,7 +13693,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="204" spans="1:16">
+    <row r="204" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
         <v>760</v>
       </c>
@@ -13691,7 +13722,7 @@
         <v>23</v>
       </c>
       <c r="J204" s="1">
-        <v>226.0</v>
+        <v>226</v>
       </c>
       <c r="K204" t="s">
         <v>41</v>
@@ -13712,7 +13743,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="205" spans="1:16">
+    <row r="205" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
         <v>765</v>
       </c>
@@ -13762,7 +13793,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="206" spans="1:16">
+    <row r="206" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>769</v>
       </c>
@@ -13812,7 +13843,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="207" spans="1:16">
+    <row r="207" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>769</v>
       </c>
@@ -13841,7 +13872,7 @@
         <v>23</v>
       </c>
       <c r="J207" s="1">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="K207" t="s">
         <v>41</v>
@@ -13862,7 +13893,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="208" spans="1:16">
+    <row r="208" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>775</v>
       </c>
@@ -13891,7 +13922,7 @@
         <v>23</v>
       </c>
       <c r="J208" s="1">
-        <v>36.3</v>
+        <v>36.299999999999997</v>
       </c>
       <c r="K208" t="s">
         <v>24</v>
@@ -13912,7 +13943,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="209" spans="1:16">
+    <row r="209" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>780</v>
       </c>
@@ -13962,7 +13993,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="210" spans="1:16">
+    <row r="210" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>784</v>
       </c>
@@ -13991,7 +14022,7 @@
         <v>23</v>
       </c>
       <c r="J210" s="1">
-        <v>21.0</v>
+        <v>21</v>
       </c>
       <c r="K210" t="s">
         <v>41</v>
@@ -14012,7 +14043,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="211" spans="1:16">
+    <row r="211" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>789</v>
       </c>
@@ -14062,7 +14093,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="212" spans="1:16">
+    <row r="212" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>793</v>
       </c>
@@ -14091,7 +14122,7 @@
         <v>23</v>
       </c>
       <c r="J212" s="1">
-        <v>286.0</v>
+        <v>286</v>
       </c>
       <c r="K212" t="s">
         <v>41</v>
@@ -14112,7 +14143,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="213" spans="1:16">
+    <row r="213" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>793</v>
       </c>
@@ -14141,7 +14172,7 @@
         <v>23</v>
       </c>
       <c r="J213" s="1">
-        <v>81.0</v>
+        <v>81</v>
       </c>
       <c r="K213" t="s">
         <v>41</v>
@@ -14162,7 +14193,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="214" spans="1:16">
+    <row r="214" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>793</v>
       </c>
@@ -14191,7 +14222,7 @@
         <v>23</v>
       </c>
       <c r="J214" s="1">
-        <v>210.0</v>
+        <v>210</v>
       </c>
       <c r="K214" t="s">
         <v>41</v>
@@ -14212,7 +14243,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="215" spans="1:16">
+    <row r="215" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>793</v>
       </c>
@@ -14241,7 +14272,7 @@
         <v>23</v>
       </c>
       <c r="J215" s="1">
-        <v>175.0</v>
+        <v>175</v>
       </c>
       <c r="K215" t="s">
         <v>41</v>
@@ -14262,7 +14293,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="216" spans="1:16">
+    <row r="216" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>806</v>
       </c>
@@ -14312,7 +14343,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="217" spans="1:16">
+    <row r="217" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>810</v>
       </c>
@@ -14341,7 +14372,7 @@
         <v>23</v>
       </c>
       <c r="J217" s="1">
-        <v>44.0</v>
+        <v>44</v>
       </c>
       <c r="K217" t="s">
         <v>24</v>
@@ -14362,7 +14393,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="218" spans="1:16">
+    <row r="218" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>815</v>
       </c>
@@ -14391,7 +14422,7 @@
         <v>23</v>
       </c>
       <c r="J218" s="1">
-        <v>56.0</v>
+        <v>56</v>
       </c>
       <c r="K218" t="s">
         <v>24</v>
@@ -14412,7 +14443,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="219" spans="1:16">
+    <row r="219" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>815</v>
       </c>
@@ -14462,7 +14493,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="220" spans="1:16">
+    <row r="220" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>815</v>
       </c>
@@ -14512,7 +14543,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="221" spans="1:16">
+    <row r="221" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>820</v>
       </c>
@@ -14541,7 +14572,7 @@
         <v>23</v>
       </c>
       <c r="J221" s="1">
-        <v>220.0</v>
+        <v>220</v>
       </c>
       <c r="K221" t="s">
         <v>41</v>
@@ -14562,7 +14593,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="222" spans="1:16">
+    <row r="222" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>825</v>
       </c>
@@ -14612,7 +14643,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="223" spans="1:16">
+    <row r="223" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>829</v>
       </c>
@@ -14662,7 +14693,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="224" spans="1:16">
+    <row r="224" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>833</v>
       </c>
@@ -14691,7 +14722,7 @@
         <v>23</v>
       </c>
       <c r="J224" s="1">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="K224" t="s">
         <v>41</v>
@@ -14712,7 +14743,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="225" spans="1:16">
+    <row r="225" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>838</v>
       </c>
@@ -14762,7 +14793,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="226" spans="1:16">
+    <row r="226" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>842</v>
       </c>
@@ -14791,7 +14822,7 @@
         <v>23</v>
       </c>
       <c r="J226" s="1">
-        <v>61.0</v>
+        <v>61</v>
       </c>
       <c r="K226" t="s">
         <v>24</v>
@@ -14812,7 +14843,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="227" spans="1:16">
+    <row r="227" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>847</v>
       </c>
@@ -14862,7 +14893,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="228" spans="1:16">
+    <row r="228" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
         <v>851</v>
       </c>
@@ -14912,7 +14943,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="229" spans="1:16">
+    <row r="229" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
         <v>855</v>
       </c>
@@ -14941,7 +14972,7 @@
         <v>23</v>
       </c>
       <c r="J229" s="1">
-        <v>11.0</v>
+        <v>11</v>
       </c>
       <c r="K229" t="s">
         <v>41</v>
@@ -14962,7 +14993,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="230" spans="1:16">
+    <row r="230" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>860</v>
       </c>
@@ -15012,7 +15043,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="231" spans="1:16">
+    <row r="231" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>864</v>
       </c>
@@ -15062,7 +15093,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="232" spans="1:16">
+    <row r="232" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
         <v>868</v>
       </c>
@@ -15112,7 +15143,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="233" spans="1:16">
+    <row r="233" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
         <v>872</v>
       </c>
@@ -15162,7 +15193,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="234" spans="1:16">
+    <row r="234" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
         <v>876</v>
       </c>
@@ -15212,7 +15243,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="235" spans="1:16">
+    <row r="235" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
         <v>876</v>
       </c>
@@ -15241,7 +15272,7 @@
         <v>23</v>
       </c>
       <c r="J235" s="1">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="K235" t="s">
         <v>41</v>
@@ -15262,7 +15293,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="236" spans="1:16">
+    <row r="236" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
         <v>882</v>
       </c>
@@ -15312,7 +15343,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="237" spans="1:16">
+    <row r="237" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
         <v>887</v>
       </c>
@@ -15341,7 +15372,7 @@
         <v>23</v>
       </c>
       <c r="J237" s="1">
-        <v>56.0</v>
+        <v>56</v>
       </c>
       <c r="K237" t="s">
         <v>24</v>
@@ -15362,7 +15393,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="238" spans="1:16">
+    <row r="238" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
         <v>887</v>
       </c>
@@ -15412,7 +15443,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="239" spans="1:16">
+    <row r="239" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
         <v>891</v>
       </c>
@@ -15462,7 +15493,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="240" spans="1:16">
+    <row r="240" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
         <v>896</v>
       </c>
@@ -15491,7 +15522,7 @@
         <v>23</v>
       </c>
       <c r="J240" s="1">
-        <v>71.4</v>
+        <v>71.400000000000006</v>
       </c>
       <c r="K240" t="s">
         <v>24</v>
@@ -15512,7 +15543,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="241" spans="1:16">
+    <row r="241" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A241" t="s">
         <v>900</v>
       </c>
@@ -15562,7 +15593,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="242" spans="1:16">
+    <row r="242" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
         <v>905</v>
       </c>
@@ -15591,7 +15622,7 @@
         <v>23</v>
       </c>
       <c r="J242" s="1">
-        <v>113.0</v>
+        <v>113</v>
       </c>
       <c r="K242" t="s">
         <v>260</v>
@@ -15612,7 +15643,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="243" spans="1:16">
+    <row r="243" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
         <v>905</v>
       </c>
@@ -15641,7 +15672,7 @@
         <v>23</v>
       </c>
       <c r="J243" s="1">
-        <v>236.0</v>
+        <v>236</v>
       </c>
       <c r="K243" t="s">
         <v>41</v>
@@ -15662,7 +15693,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="244" spans="1:16">
+    <row r="244" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>912</v>
       </c>
@@ -15691,7 +15722,7 @@
         <v>23</v>
       </c>
       <c r="J244" s="1">
-        <v>162.0</v>
+        <v>162</v>
       </c>
       <c r="K244" t="s">
         <v>41</v>
@@ -15712,7 +15743,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="245" spans="1:16">
+    <row r="245" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>912</v>
       </c>
@@ -15741,7 +15772,7 @@
         <v>23</v>
       </c>
       <c r="J245" s="1">
-        <v>91.0</v>
+        <v>91</v>
       </c>
       <c r="K245" t="s">
         <v>41</v>
@@ -15762,7 +15793,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="246" spans="1:16">
+    <row r="246" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A246" t="s">
         <v>919</v>
       </c>
@@ -15812,7 +15843,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="247" spans="1:16">
+    <row r="247" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
         <v>923</v>
       </c>
@@ -15862,7 +15893,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="248" spans="1:16">
+    <row r="248" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
         <v>927</v>
       </c>
@@ -15912,7 +15943,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="249" spans="1:16">
+    <row r="249" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
         <v>931</v>
       </c>
@@ -15941,7 +15972,7 @@
         <v>23</v>
       </c>
       <c r="J249" s="1">
-        <v>392.0</v>
+        <v>392</v>
       </c>
       <c r="K249" t="s">
         <v>41</v>
@@ -15962,7 +15993,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="250" spans="1:16">
+    <row r="250" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
         <v>936</v>
       </c>
@@ -15991,7 +16022,7 @@
         <v>23</v>
       </c>
       <c r="J250" s="1">
-        <v>119.0</v>
+        <v>119</v>
       </c>
       <c r="K250" t="s">
         <v>41</v>
@@ -16012,7 +16043,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="251" spans="1:16">
+    <row r="251" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
         <v>936</v>
       </c>
@@ -16041,7 +16072,7 @@
         <v>23</v>
       </c>
       <c r="J251" s="1">
-        <v>620.0</v>
+        <v>620</v>
       </c>
       <c r="K251" t="s">
         <v>41</v>
@@ -16062,7 +16093,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="252" spans="1:16">
+    <row r="252" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
         <v>943</v>
       </c>
@@ -16091,7 +16122,7 @@
         <v>23</v>
       </c>
       <c r="J252" s="1">
-        <v>48.0</v>
+        <v>48</v>
       </c>
       <c r="K252" t="s">
         <v>24</v>
@@ -16112,7 +16143,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="253" spans="1:16">
+    <row r="253" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A253" t="s">
         <v>948</v>
       </c>
@@ -16141,7 +16172,7 @@
         <v>23</v>
       </c>
       <c r="J253" s="1">
-        <v>126.0</v>
+        <v>126</v>
       </c>
       <c r="K253" t="s">
         <v>41</v>
@@ -16162,7 +16193,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="254" spans="1:16">
+    <row r="254" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
         <v>948</v>
       </c>
@@ -16191,7 +16222,7 @@
         <v>23</v>
       </c>
       <c r="J254" s="1">
-        <v>161.0</v>
+        <v>161</v>
       </c>
       <c r="K254" t="s">
         <v>41</v>
@@ -16212,7 +16243,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="255" spans="1:16">
+    <row r="255" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
         <v>955</v>
       </c>
@@ -16262,7 +16293,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="256" spans="1:16">
+    <row r="256" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A256" t="s">
         <v>960</v>
       </c>
@@ -16291,7 +16322,7 @@
         <v>23</v>
       </c>
       <c r="J256" s="1">
-        <v>231.0</v>
+        <v>231</v>
       </c>
       <c r="K256" t="s">
         <v>41</v>
@@ -16312,7 +16343,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="257" spans="1:16">
+    <row r="257" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
         <v>965</v>
       </c>
@@ -16341,7 +16372,7 @@
         <v>23</v>
       </c>
       <c r="J257" s="1">
-        <v>256.0</v>
+        <v>256</v>
       </c>
       <c r="K257" t="s">
         <v>41</v>
@@ -16362,7 +16393,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="258" spans="1:16">
+    <row r="258" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A258" t="s">
         <v>968</v>
       </c>
@@ -16391,7 +16422,7 @@
         <v>23</v>
       </c>
       <c r="J258" s="1">
-        <v>176.0</v>
+        <v>176</v>
       </c>
       <c r="K258" t="s">
         <v>41</v>
@@ -16412,7 +16443,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="259" spans="1:16">
+    <row r="259" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A259" t="s">
         <v>973</v>
       </c>
@@ -16441,7 +16472,7 @@
         <v>23</v>
       </c>
       <c r="J259" s="1">
-        <v>17.0</v>
+        <v>17</v>
       </c>
       <c r="K259" t="s">
         <v>41</v>
@@ -16462,7 +16493,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="260" spans="1:16">
+    <row r="260" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
         <v>978</v>
       </c>
@@ -16512,7 +16543,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="261" spans="1:16">
+    <row r="261" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A261" t="s">
         <v>983</v>
       </c>
@@ -16541,7 +16572,7 @@
         <v>23</v>
       </c>
       <c r="J261" s="1">
-        <v>75.4</v>
+        <v>75.400000000000006</v>
       </c>
       <c r="K261" t="s">
         <v>24</v>
@@ -16562,7 +16593,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="262" spans="1:16">
+    <row r="262" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A262" t="s">
         <v>983</v>
       </c>
@@ -16591,7 +16622,7 @@
         <v>23</v>
       </c>
       <c r="J262" s="1">
-        <v>11.0</v>
+        <v>11</v>
       </c>
       <c r="K262" t="s">
         <v>41</v>
@@ -16612,7 +16643,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="263" spans="1:16">
+    <row r="263" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A263" t="s">
         <v>989</v>
       </c>
@@ -16641,7 +16672,7 @@
         <v>23</v>
       </c>
       <c r="J263" s="1">
-        <v>75.4</v>
+        <v>75.400000000000006</v>
       </c>
       <c r="K263" t="s">
         <v>24</v>
@@ -16662,7 +16693,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="264" spans="1:16">
+    <row r="264" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
         <v>993</v>
       </c>
@@ -16712,7 +16743,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="265" spans="1:16">
+    <row r="265" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
         <v>998</v>
       </c>
@@ -16762,7 +16793,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="266" spans="1:16">
+    <row r="266" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A266" t="s">
         <v>1002</v>
       </c>
@@ -16791,7 +16822,7 @@
         <v>23</v>
       </c>
       <c r="J266" s="1">
-        <v>71.0</v>
+        <v>71</v>
       </c>
       <c r="K266" t="s">
         <v>260</v>
@@ -16812,7 +16843,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="267" spans="1:16">
+    <row r="267" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A267" t="s">
         <v>1002</v>
       </c>
@@ -16841,7 +16872,7 @@
         <v>23</v>
       </c>
       <c r="J267" s="1">
-        <v>184.0</v>
+        <v>184</v>
       </c>
       <c r="K267" t="s">
         <v>260</v>
@@ -16862,7 +16893,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="268" spans="1:16">
+    <row r="268" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A268" t="s">
         <v>1002</v>
       </c>
@@ -16891,7 +16922,7 @@
         <v>23</v>
       </c>
       <c r="J268" s="1">
-        <v>95.0</v>
+        <v>95</v>
       </c>
       <c r="K268" t="s">
         <v>260</v>
@@ -16912,7 +16943,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="269" spans="1:16">
+    <row r="269" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A269" t="s">
         <v>1012</v>
       </c>
@@ -16962,7 +16993,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="270" spans="1:16">
+    <row r="270" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A270" t="s">
         <v>1016</v>
       </c>
@@ -17012,7 +17043,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="271" spans="1:16">
+    <row r="271" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A271" t="s">
         <v>1020</v>
       </c>
@@ -17062,7 +17093,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="272" spans="1:16">
+    <row r="272" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A272" t="s">
         <v>1024</v>
       </c>
@@ -17112,7 +17143,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="273" spans="1:16">
+    <row r="273" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A273" t="s">
         <v>1028</v>
       </c>
@@ -17162,7 +17193,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="274" spans="1:16">
+    <row r="274" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A274" t="s">
         <v>1028</v>
       </c>
@@ -17191,7 +17222,7 @@
         <v>23</v>
       </c>
       <c r="J274" s="1">
-        <v>277.0</v>
+        <v>277</v>
       </c>
       <c r="K274" t="s">
         <v>41</v>
@@ -17212,7 +17243,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="275" spans="1:16">
+    <row r="275" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A275" t="s">
         <v>1028</v>
       </c>
@@ -17241,7 +17272,7 @@
         <v>23</v>
       </c>
       <c r="J275" s="1">
-        <v>21.0</v>
+        <v>21</v>
       </c>
       <c r="K275" t="s">
         <v>41</v>
@@ -17262,7 +17293,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="276" spans="1:16">
+    <row r="276" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A276" t="s">
         <v>1036</v>
       </c>
@@ -17291,7 +17322,7 @@
         <v>23</v>
       </c>
       <c r="J276" s="1">
-        <v>73.0</v>
+        <v>73</v>
       </c>
       <c r="K276" t="s">
         <v>24</v>
@@ -17312,7 +17343,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="277" spans="1:16">
+    <row r="277" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A277" t="s">
         <v>1036</v>
       </c>
@@ -17341,7 +17372,7 @@
         <v>23</v>
       </c>
       <c r="J277" s="1">
-        <v>421.0</v>
+        <v>421</v>
       </c>
       <c r="K277" t="s">
         <v>41</v>
@@ -17362,7 +17393,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="278" spans="1:16">
+    <row r="278" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A278" t="s">
         <v>1036</v>
       </c>
@@ -17391,7 +17422,7 @@
         <v>23</v>
       </c>
       <c r="J278" s="1">
-        <v>677.0</v>
+        <v>677</v>
       </c>
       <c r="K278" t="s">
         <v>41</v>
@@ -17412,7 +17443,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="279" spans="1:16">
+    <row r="279" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A279" t="s">
         <v>1044</v>
       </c>
@@ -17462,7 +17493,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="280" spans="1:16">
+    <row r="280" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A280" t="s">
         <v>1044</v>
       </c>
@@ -17512,7 +17543,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="281" spans="1:16">
+    <row r="281" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A281" t="s">
         <v>1048</v>
       </c>
@@ -17562,7 +17593,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="282" spans="1:16">
+    <row r="282" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A282" t="s">
         <v>1052</v>
       </c>
@@ -17591,7 +17622,7 @@
         <v>23</v>
       </c>
       <c r="J282" s="1">
-        <v>71.4</v>
+        <v>71.400000000000006</v>
       </c>
       <c r="K282" t="s">
         <v>24</v>
@@ -17613,17 +17644,13 @@
       </c>
     </row>
   </sheetData>
-  <printOptions gridLines="false" gridLinesSet="true"/>
+  <autoFilter ref="A1:P282" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="5">
+      <filters>
+        <filter val="byt"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
-  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddHeader/>
-    <oddFooter/>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
-  <tableParts count="0"/>
 </worksheet>
 </file>
</xml_diff>